<commit_message>
Footing Jacket workbook: add the locked Theory sheet
Sheet 2 sets out the equations behind each section of the calculation
sheet as locked pictures, with the clause and printed page under each.
They are typeset for the workbook, not copied from the standards.
Rebuilt from apec-cfrp-beam excel/ (theory.py); the calculation sheet is
unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/APEC-Footing-Jacket.xlsx
+++ b/excel/APEC-Footing-Jacket.xlsx
@@ -8,10 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Footing Jacket" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Theory" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Footing Jacket'!$9:$9</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Footing Jacket'!$B$1:$G$349</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Theory'!$9:$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Theory'!$B$1:$G$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -164,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -289,6 +292,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -467,6 +476,308 @@
         <a:xfrm>
           <a:off x="1943100" y="2406650"/>
           <a:ext cx="7239000" cy="3286125"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>342900</colOff>
+      <row>0</row>
+      <rowOff>114300</rowOff>
+    </from>
+    <ext cx="3476625" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="476250" y="114300"/>
+          <a:ext cx="3476625" cy="685800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>1809750</colOff>
+      <row>12</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="7239000" cy="2266950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1943100" y="2736850"/>
+          <a:ext cx="7239000" cy="2266950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>1809750</colOff>
+      <row>29</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="7239000" cy="2095500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1943100" y="5988050"/>
+          <a:ext cx="7239000" cy="2095500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>1809750</colOff>
+      <row>45</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="7239000" cy="1885950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1943100" y="9048750"/>
+          <a:ext cx="7239000" cy="1885950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>1809750</colOff>
+      <row>60</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="7239000" cy="1057275"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1943100" y="12084050"/>
+          <a:ext cx="7239000" cy="1057275"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>1809750</colOff>
+      <row>71</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="7239000" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1943100" y="14192250"/>
+          <a:ext cx="7239000" cy="2047875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>1809750</colOff>
+      <row>87</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="7239000" cy="1552575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1943100" y="17418050"/>
+          <a:ext cx="7239000" cy="1552575"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>1809750</colOff>
+      <row>100</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="7239000" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1943100" y="19907250"/>
+          <a:ext cx="7239000" cy="2047875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>1809750</colOff>
+      <row>116</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="7239000" cy="1885950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1943100" y="23133050"/>
+          <a:ext cx="7239000" cy="1885950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2034,7 +2345,7 @@
     <row r="85" ht="13" customHeight="1">
       <c r="B85" s="22" t="inlineStr">
         <is>
-          <t>Background on footing strengthening and why it is rarely straightforward: Antoniou (2023), Section 4.18.</t>
+          <t>Background on footing strengthening and why it is rarely straightforward: Antoniou (2023), Section 4.18. The equations behind each section, with clause and page, are on the Theory sheet.</t>
         </is>
       </c>
     </row>
@@ -7423,4 +7734,427 @@
   </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G131"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>D E S I G N    S H E E T</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Project :</t>
+        </is>
+      </c>
+      <c r="E2" s="44" t="str">
+        <f>'Footing Jacket'!$E$2</f>
+        <v>Project name</v>
+      </c>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Member :</t>
+        </is>
+      </c>
+      <c r="E3" s="44" t="str">
+        <f>'Footing Jacket'!$E$3</f>
+        <v>F-1 - Grid A-1</v>
+      </c>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Designed / Date :</t>
+        </is>
+      </c>
+      <c r="E4" s="44" t="str">
+        <f>'Footing Jacket'!$E$4</f>
+        <v>APEC</v>
+      </c>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="45">
+        <f>'Footing Jacket'!$G$4</f>
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>THEORETICAL REFERENCE - FOOTING JACKET</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>ACI 562-25; ACI 318-25M; ASCE 41-17 - clause and printed page under each card</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Reference sheet - no inputs. Every cell and picture is locked. Owner: Albert Pamonag - Albert Pamonag Engineering Consultancy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Equations and provisions behind the calculation sheet</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>Each card sets out, in this sheet's own notation, the equations a section of the calculation sheet uses; the line under it gives the clause and the printed page where the provision is found. The cards are typeset for this workbook - they are not copies of the standards, which remain the authority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>A.  LOAD HISTORY AND BEARING PRESSURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1"/>
+    <row r="14" ht="15" customHeight="1"/>
+    <row r="15" ht="15" customHeight="1"/>
+    <row r="16" ht="15" customHeight="1"/>
+    <row r="17" ht="15" customHeight="1"/>
+    <row r="18" ht="15" customHeight="1"/>
+    <row r="19" ht="15" customHeight="1"/>
+    <row r="20" ht="15" customHeight="1"/>
+    <row r="21" ht="15" customHeight="1"/>
+    <row r="22" ht="15" customHeight="1"/>
+    <row r="23" ht="15" customHeight="1"/>
+    <row r="24" ht="15" customHeight="1"/>
+    <row r="25" ht="15" customHeight="1"/>
+    <row r="26" ht="15" customHeight="1"/>
+    <row r="27" ht="13" customHeight="1">
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>Basis: ACI 562-25 R9.4.1 (p. 85) and R9.2.1 (p. 84); ASCE 41-17 C8.7 item 2 (p. 455); ACI 318-25M 13.3.1.1 (p. 211).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29" ht="18" customHeight="1">
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>B.  PRESSURE BEYOND A SECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31" ht="15" customHeight="1"/>
+    <row r="32" ht="15" customHeight="1"/>
+    <row r="33" ht="15" customHeight="1"/>
+    <row r="34" ht="15" customHeight="1"/>
+    <row r="35" ht="15" customHeight="1"/>
+    <row r="36" ht="15" customHeight="1"/>
+    <row r="37" ht="15" customHeight="1"/>
+    <row r="38" ht="15" customHeight="1"/>
+    <row r="39" ht="15" customHeight="1"/>
+    <row r="40" ht="15" customHeight="1"/>
+    <row r="41" ht="15" customHeight="1"/>
+    <row r="42" ht="15" customHeight="1"/>
+    <row r="43" ht="13" customHeight="1">
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>Basis: Statics. Critical sections: ACI 318-25M Table 13.2.7.1 and 13.2.7.2 (p. 210), 7.4.3.2 (p. 101).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45" ht="18" customHeight="1">
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>C.  FLEXURE OF THE COMPOSITE SECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15" customHeight="1"/>
+    <row r="47" ht="15" customHeight="1"/>
+    <row r="48" ht="15" customHeight="1"/>
+    <row r="49" ht="15" customHeight="1"/>
+    <row r="50" ht="15" customHeight="1"/>
+    <row r="51" ht="15" customHeight="1"/>
+    <row r="52" ht="15" customHeight="1"/>
+    <row r="53" ht="15" customHeight="1"/>
+    <row r="54" ht="15" customHeight="1"/>
+    <row r="55" ht="15" customHeight="1"/>
+    <row r="56" ht="15" customHeight="1"/>
+    <row r="57" ht="15" customHeight="1"/>
+    <row r="58" ht="26" customHeight="1">
+      <c r="B58" s="22" t="inlineStr">
+        <is>
+          <t>Basis: ACI 318-25M 22.3.3.2 to 22.3.3.4 (p. 440), Table 22.2.2.4.3 (p. 439), 7.6.1.1 (p. 102), 8.6.1.1 (p. 122), 13.3.1.2 (p. 212); ACI 562-25 Table 5.3.2 (p. 38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59"/>
+    <row r="60" ht="18" customHeight="1">
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>D.  ONE-WAY SHEAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15" customHeight="1"/>
+    <row r="62" ht="15" customHeight="1"/>
+    <row r="63" ht="15" customHeight="1"/>
+    <row r="64" ht="15" customHeight="1"/>
+    <row r="65" ht="15" customHeight="1"/>
+    <row r="66" ht="15" customHeight="1"/>
+    <row r="67" ht="15" customHeight="1"/>
+    <row r="68" ht="15" customHeight="1"/>
+    <row r="69" ht="13" customHeight="1">
+      <c r="B69" s="22" t="inlineStr">
+        <is>
+          <t>Basis: ACI 318-25M 13.2.6.2(a) (p. 208), 22.5.3.1 (p. 443), 22.5.4.2 to 22.5.4.4 (p. 444); ACI 562-25 Table 5.3.2 (p. 38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70"/>
+    <row r="71" ht="18" customHeight="1">
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t>E.  TWO-WAY SHEAR WITH MOMENT TRANSFER</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="15" customHeight="1"/>
+    <row r="73" ht="15" customHeight="1"/>
+    <row r="74" ht="15" customHeight="1"/>
+    <row r="75" ht="15" customHeight="1"/>
+    <row r="76" ht="15" customHeight="1"/>
+    <row r="77" ht="15" customHeight="1"/>
+    <row r="78" ht="15" customHeight="1"/>
+    <row r="79" ht="15" customHeight="1"/>
+    <row r="80" ht="15" customHeight="1"/>
+    <row r="81" ht="15" customHeight="1"/>
+    <row r="82" ht="15" customHeight="1"/>
+    <row r="83" ht="15" customHeight="1"/>
+    <row r="84" ht="15" customHeight="1"/>
+    <row r="85" ht="26" customHeight="1">
+      <c r="B85" s="22" t="inlineStr">
+        <is>
+          <t>Basis: ACI 318-25M 22.6.4.1 (p. 451), Table 22.6.5.2 (p. 454), 22.6.5.3 (p. 455), 13.2.6.2(b) (p. 208), Eq. 8.4.2.2.2 (p. 116), 8.4.4.2 and R8.4.4.2.3 (p. 118-119).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86"/>
+    <row r="87" ht="18" customHeight="1">
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>F.  MINIMUM REINFORCEMENT AT THE COLUMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="15" customHeight="1"/>
+    <row r="89" ht="15" customHeight="1"/>
+    <row r="90" ht="15" customHeight="1"/>
+    <row r="91" ht="15" customHeight="1"/>
+    <row r="92" ht="15" customHeight="1"/>
+    <row r="93" ht="15" customHeight="1"/>
+    <row r="94" ht="15" customHeight="1"/>
+    <row r="95" ht="15" customHeight="1"/>
+    <row r="96" ht="15" customHeight="1"/>
+    <row r="97" ht="15" customHeight="1"/>
+    <row r="98" ht="13" customHeight="1">
+      <c r="B98" s="22" t="inlineStr">
+        <is>
+          <t>Basis: ACI 318-25M Eq. 8.6.1.2 (p. 122), 8.4.2.2.3 (p. 116-117), Eq. 22.5.5.1.3 (p. 445).</t>
+        </is>
+      </c>
+    </row>
+    <row r="99"/>
+    <row r="100" ht="18" customHeight="1">
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>G.  SHEAR FRICTION ON THE OLD FACES</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1"/>
+    <row r="102" ht="15" customHeight="1"/>
+    <row r="103" ht="15" customHeight="1"/>
+    <row r="104" ht="15" customHeight="1"/>
+    <row r="105" ht="15" customHeight="1"/>
+    <row r="106" ht="15" customHeight="1"/>
+    <row r="107" ht="15" customHeight="1"/>
+    <row r="108" ht="15" customHeight="1"/>
+    <row r="109" ht="15" customHeight="1"/>
+    <row r="110" ht="15" customHeight="1"/>
+    <row r="111" ht="15" customHeight="1"/>
+    <row r="112" ht="15" customHeight="1"/>
+    <row r="113" ht="15" customHeight="1"/>
+    <row r="114" ht="26" customHeight="1">
+      <c r="B114" s="22" t="inlineStr">
+        <is>
+          <t>Basis: ACI 318-25M Eq. 22.9.4.2 and Table 22.9.4.2 (p. 472), Table 22.9.4.4 (p. 474), Table 20.2.2.4(a) (p. 414), 22.3.3.1 (p. 440); ACI 562-25 9.4.4.3 (p. 89), R9.4.5.3 (p. 90), Table 5.3.2 (p. 38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="115"/>
+    <row r="116" ht="18" customHeight="1">
+      <c r="B116" s="10" t="inlineStr">
+        <is>
+          <t>H.  HORIZONTAL SHEAR UNDER THE OVERLAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="15" customHeight="1"/>
+    <row r="118" ht="15" customHeight="1"/>
+    <row r="119" ht="15" customHeight="1"/>
+    <row r="120" ht="15" customHeight="1"/>
+    <row r="121" ht="15" customHeight="1"/>
+    <row r="122" ht="15" customHeight="1"/>
+    <row r="123" ht="15" customHeight="1"/>
+    <row r="124" ht="15" customHeight="1"/>
+    <row r="125" ht="15" customHeight="1"/>
+    <row r="126" ht="15" customHeight="1"/>
+    <row r="127" ht="15" customHeight="1"/>
+    <row r="128" ht="15" customHeight="1"/>
+    <row r="129" ht="13" customHeight="1">
+      <c r="B129" s="22" t="inlineStr">
+        <is>
+          <t>Basis: ACI 318-25M 16.4.1.2 and Eq. 16.4.3.1 (p. 243), Table 16.4.4.1 (p. 244), 16.4.6.1 and 16.4.7.2 (p. 246).</t>
+        </is>
+      </c>
+    </row>
+    <row r="130"/>
+    <row r="131" ht="26" customHeight="1">
+      <c r="B131" s="22" t="inlineStr">
+        <is>
+          <t>(c) Albert Pamonag Engineering Consultancy. Owner: Albert Pamonag. This calculation sheet is protected; the engineer of record remains responsible for the inputs and for the checks listed as not covered.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="EC33"/>
+  <mergeCells count="27">
+    <mergeCell ref="B60:G60"/>
+    <mergeCell ref="B98:G98"/>
+    <mergeCell ref="B1:C4"/>
+    <mergeCell ref="B116:G116"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B69:G69"/>
+    <mergeCell ref="B87:G87"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B85:G85"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B114:G114"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="B100:G100"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B129:G129"/>
+    <mergeCell ref="B131:G131"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B71:G71"/>
+    <mergeCell ref="B43:G43"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B58:G58"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G10:G130">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"PASS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>"FAIL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
+      <formula>"INVALID INPUT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
+      <formula>"NO ROOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2">
+      <formula>"WARN"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="2">
+      <formula>"CHECK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="2">
+      <formula>"OVERRIDE"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="2">
+      <formula>"NOT CHECKED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="2">
+      <formula>"CAPPED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="2">
+      <formula>"REDUCED"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;8 (c) Albert Pamonag Engineering Consultancy - Owner: Albert Pamonag&amp;C&amp;8 &amp;A&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>